<commit_message>
🐛 fix: fixed hotel xansha templates
</commit_message>
<xml_diff>
--- a/apps/excel-service/templates/XANSHA/HOTEL/Completed Work Certificates.xlsx
+++ b/apps/excel-service/templates/XANSHA/HOTEL/Completed Work Certificates.xlsx
@@ -1008,7 +1008,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr defaultColWidth="16.829999999999998" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -52124,8 +52124,8 @@
     <mergeCell ref="AL40:AQ40"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0" footer="0"/>
+  <pageSetup paperSize="9" scale="91" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
</xml_diff>